<commit_message>
Cambios sustanciales en Muestra (filtrados por calles) y recálculo de todo.
</commit_message>
<xml_diff>
--- a/Output/Tables/Outcomes_by_PHC_org.xlsx
+++ b/Output/Tables/Outcomes_by_PHC_org.xlsx
@@ -351,27 +351,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>[ALL]   N=2058</t>
+          <t>[ALL]   N=1963</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Equip_Atdom   N=743</t>
+          <t>Equip_Atdom   N=714</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Equip_Inf   N=299</t>
+          <t>Equip_Inf   N=260</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>UAB_consulta   N=367</t>
+          <t>UAB_consulta   N=353</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>UAB_consulta_reforc   N=649</t>
+          <t>UAB_consulta_reforc   N=636</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -487,7 +487,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.001  </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CAMBIOS IMPORTANTES EN MUESTRA TOTAL Y RESTRUTURA DE ANÁLISIS
</commit_message>
<xml_diff>
--- a/Output/Tables/Outcomes_by_PHC_org.xlsx
+++ b/Output/Tables/Outcomes_by_PHC_org.xlsx
@@ -340,7 +340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -351,27 +351,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>[ALL]   N=1963</t>
+          <t>[ALL]   N=1338</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Equip_Atdom   N=714</t>
+          <t>Equip_Atdom   N=491</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Equip_Inf   N=260</t>
+          <t>Equip_Inf   N=199</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>UAB_consulta   N=353</t>
+          <t>UAB_consulta   N=253</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>UAB_consulta_reforc   N=636</t>
+          <t>UAB_consulta_reforc   N=395</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -383,44 +383,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SEM_num, Median [25th;75th]</t>
+          <t>Home_Ambulances, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.00 [0.00;2.00]</t>
+          <t>1.00 [1.00;3.00]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.00 [0.00;2.00]</t>
+          <t>2.00 [1.00;3.00]</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.00 [0.00;2.00]</t>
+          <t>2.00 [1.00;3.00]</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.00 [0.00;2.00]</t>
+          <t>2.00 [1.00;3.00]</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.00 [0.00;2.00]  </t>
+          <t xml:space="preserve"> 1.00 [1.00;3.00]  </t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.002  </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>emergency_visits, Median [25th;75th]</t>
+          <t>ED_visits, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -445,19 +445,19 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.00 [0.00;2.00]  </t>
+          <t xml:space="preserve"> 1.00 [0.00;2.00]  </t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.001  </t>
+          <t xml:space="preserve">  0.366  </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INGRES_num, Median [25th;75th]</t>
+          <t>PC_Emergency_visits, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -487,7 +487,44 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.001  </t>
+          <t xml:space="preserve">  0.102  </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hospital_Admissions, Median [25th;75th]</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1.00 [0.00;1.00]</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.00 [0.00;1.00]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1.00 [0.00;2.00]</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.00 [0.00;1.00]</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 0.00 [0.00;1.00]  </t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  0.031  </t>
         </is>
       </c>
     </row>

</xml_diff>